<commit_message>
update work and file formats
</commit_message>
<xml_diff>
--- a/src/docs/excel_templates/employee_attendance.xlsx
+++ b/src/docs/excel_templates/employee_attendance.xlsx
@@ -27,10 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
-  <si>
-    <t>Template Columns</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Employee Code</t>
   </si>
@@ -680,9 +677,8 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1025,84 +1021,79 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8" outlineLevelCol="6"/>
   <cols>
     <col min="1" max="1" width="16.6666666666667" customWidth="1"/>
     <col min="2" max="2" width="15.225" customWidth="1"/>
-    <col min="3" max="3" width="14.3333333333333" customWidth="1"/>
-    <col min="4" max="4" width="11" customWidth="1"/>
-    <col min="5" max="5" width="7.44166666666667" customWidth="1"/>
-    <col min="6" max="6" width="11" customWidth="1"/>
+    <col min="3" max="3" width="15.8" customWidth="1"/>
+    <col min="4" max="4" width="7.9" customWidth="1"/>
+    <col min="5" max="5" width="8.3" customWidth="1"/>
+    <col min="6" max="6" width="9.4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:1">
+    <row r="1" s="1" customFormat="1" spans="1:7">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" s="1" customFormat="1" spans="1:7">
-      <c r="A2" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="3" t="s">
-        <v>7</v>
-      </c>
+    </row>
+    <row r="2" spans="3:6">
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="F2" s="3"/>
     </row>
     <row r="3" spans="3:6">
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="F3" s="4"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="F3" s="3"/>
     </row>
     <row r="4" spans="3:6">
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="F4" s="4"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="F4" s="3"/>
     </row>
     <row r="5" spans="3:6">
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="F5" s="4"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="F5" s="3"/>
     </row>
     <row r="6" spans="3:6">
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="F6" s="4"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="F6" s="3"/>
     </row>
     <row r="7" spans="3:6">
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="F7" s="4"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="F7" s="3"/>
     </row>
     <row r="8" spans="3:6">
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="F8" s="4"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="F8" s="3"/>
     </row>
     <row r="9" spans="3:6">
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="F9" s="4"/>
-    </row>
-    <row r="10" spans="3:6">
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="F10" s="4"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="F9" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>